<commit_message>
feat: add guideline sheet to tryout export workbook
- Generate a guideline sheet listing column definitions, required fields, and valid values for each import table.
- Display category tree branches on the evaluation page for better visual hierarchy.
- Show answer summary (correct/total) per attempt in evaluation results.
- Fix embedded YouTube URL parsing in review page.
</commit_message>
<xml_diff>
--- a/docs/ilmorax-tryout-sample.xlsx
+++ b/docs/ilmorax-tryout-sample.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="tryout" sheetId="1" r:id="rId1"/>
     <sheet name="questions" sheetId="2" r:id="rId2"/>
+    <sheet name="guideline" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -398,7 +399,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="72.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -411,12 +421,15 @@
         <v>category_id</v>
       </c>
       <c r="D1" t="str">
+        <v>category_name</v>
+      </c>
+      <c r="E1" t="str">
         <v>duration_minutes</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>access_level</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>status</v>
       </c>
     </row>
@@ -428,28 +441,50 @@
         <v>Sample Try-out description. Replace this with the real Student-facing description.</v>
       </c>
       <c r="C2" t="str">
-        <v>farmakologi</v>
-      </c>
-      <c r="D2">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v>Farmakologi</v>
+      </c>
+      <c r="E2">
         <v>30</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>free</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>draft</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:Q3"/>
+  <cols>
+    <col min="1" max="1" width="13.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="17.83203125" customWidth="1"/>
+    <col min="6" max="6" width="19.83203125" customWidth="1"/>
+    <col min="7" max="7" width="44.83203125" customWidth="1"/>
+    <col min="8" max="8" width="29.83203125" customWidth="1"/>
+    <col min="9" max="9" width="33.83203125" customWidth="1"/>
+    <col min="10" max="10" width="26.83203125" customWidth="1"/>
+    <col min="11" max="11" width="27.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="72.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -462,39 +497,45 @@
         <v>category_id</v>
       </c>
       <c r="D1" t="str">
+        <v>category_name</v>
+      </c>
+      <c r="E1" t="str">
         <v>sub_category_id</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
+        <v>sub_category_name</v>
+      </c>
+      <c r="G1" t="str">
         <v>question_text</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>option_a</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>option_b</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>option_c</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>option_d</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>option_e</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>correct_option</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>explanation</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>video_url</v>
       </c>
-      <c r="N1" t="str">
+      <c r="P1" t="str">
         <v>access_level</v>
       </c>
-      <c r="O1" t="str">
+      <c r="Q1" t="str">
         <v>status</v>
       </c>
     </row>
@@ -506,42 +547,48 @@
         <v>1</v>
       </c>
       <c r="C2" t="str">
-        <v>farmakologi</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>farmakologi-antibiotik</v>
+        <v>Farmakologi</v>
       </c>
       <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v>Antibiotik</v>
+      </c>
+      <c r="G2" t="str">
         <v>Mekanisme kerja penisilin adalah:</v>
       </c>
-      <c r="F2" t="str">
+      <c r="H2" t="str">
         <v>Menghambat sintesis protein</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v>Menghambat sintesis dinding sel</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>Menghambat replikasi DNA</v>
       </c>
-      <c r="I2" t="str">
+      <c r="K2" t="str">
         <v>Menghambat sintesis folat</v>
       </c>
-      <c r="J2" t="str">
+      <c r="L2" t="str">
         <v/>
       </c>
-      <c r="K2" t="str">
+      <c r="M2" t="str">
         <v>B</v>
       </c>
-      <c r="L2" t="str">
+      <c r="N2" t="str">
         <v>Penisilin menghambat sintesis dinding sel bakteri dengan mengikat protein pengikat penisilin.</v>
       </c>
-      <c r="M2" t="str">
+      <c r="O2" t="str">
         <v/>
       </c>
-      <c r="N2" t="str">
+      <c r="P2" t="str">
         <v>free</v>
       </c>
-      <c r="O2" t="str">
+      <c r="Q2" t="str">
         <v>draft</v>
       </c>
     </row>
@@ -553,48 +600,667 @@
         <v>2</v>
       </c>
       <c r="C3" t="str">
-        <v>farmakologi</v>
+        <v/>
       </c>
       <c r="D3" t="str">
-        <v>farmakologi-nsaid</v>
+        <v>Farmakologi</v>
       </c>
       <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>NSAID</v>
+      </c>
+      <c r="G3" t="str">
         <v>NSAID yang paling selektif terhadap COX-2:</v>
       </c>
-      <c r="F3" t="str">
+      <c r="H3" t="str">
         <v>Ibuprofen</v>
       </c>
-      <c r="G3" t="str">
+      <c r="I3" t="str">
         <v>Celecoxib</v>
       </c>
-      <c r="H3" t="str">
+      <c r="J3" t="str">
         <v>Aspirin</v>
       </c>
-      <c r="I3" t="str">
+      <c r="K3" t="str">
         <v>Diklofenak</v>
       </c>
-      <c r="J3" t="str">
+      <c r="L3" t="str">
         <v/>
       </c>
-      <c r="K3" t="str">
+      <c r="M3" t="str">
         <v>B</v>
       </c>
-      <c r="L3" t="str">
+      <c r="N3" t="str">
         <v>Celecoxib adalah NSAID selektif COX-2 yang menurunkan risiko gangguan gastrointestinal.</v>
       </c>
-      <c r="M3" t="str">
+      <c r="O3" t="str">
         <v/>
       </c>
-      <c r="N3" t="str">
+      <c r="P3" t="str">
         <v>free</v>
       </c>
-      <c r="O3" t="str">
+      <c r="Q3" t="str">
         <v>draft</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E35"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="19.83203125" customWidth="1"/>
+    <col min="3" max="3" width="42.83203125" customWidth="1"/>
+    <col min="4" max="4" width="72.83203125" customWidth="1"/>
+    <col min="5" max="5" width="72.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>sheet</v>
+      </c>
+      <c r="B1" t="str">
+        <v>column</v>
+      </c>
+      <c r="C1" t="str">
+        <v>required</v>
+      </c>
+      <c r="D1" t="str">
+        <v>possible_values</v>
+      </c>
+      <c r="E1" t="str">
+        <v>notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>tryout</v>
+      </c>
+      <c r="B2" t="str">
+        <v>title</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Any text</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Name shown to students and admins.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>tryout</v>
+      </c>
+      <c r="B3" t="str">
+        <v>description</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Any text</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Short student-facing description.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>tryout</v>
+      </c>
+      <c r="B4" t="str">
+        <v>category_id</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Use category_id or category_name</v>
+      </c>
+      <c r="D4" t="str">
+        <v>klinis, farmakologi, farmasi-klinik</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Use an existing Category ID when available.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>tryout</v>
+      </c>
+      <c r="B5" t="str">
+        <v>category_name</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Use category_id or category_name</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Klinis, Farmakologi, Farmasi Klinik or a new Category name</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Use an existing Category name or type a new one to create it during import.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>tryout</v>
+      </c>
+      <c r="B6" t="str">
+        <v>duration_minutes</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D6" t="str">
+        <v>1-300</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Whole number of minutes.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>tryout</v>
+      </c>
+      <c r="B7" t="str">
+        <v>access_level</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D7" t="str">
+        <v>free, premium</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Controls who can access this Try-out.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>tryout</v>
+      </c>
+      <c r="B8" t="str">
+        <v>status</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D8" t="str">
+        <v>draft, published, unpublished</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Use draft while preparing content.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B9" t="str">
+        <v>question_id</v>
+      </c>
+      <c r="C9" t="str">
+        <v>No</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Existing Question ID</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Leave blank to create a new Question. Use the exported ID to update an existing Question.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B10" t="str">
+        <v>sort_order</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D10" t="str">
+        <v>1-1000</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Question order inside the Try-out. Must be unique.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B11" t="str">
+        <v>category_id</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Use category_id or category_name</v>
+      </c>
+      <c r="D11" t="str">
+        <v>klinis, farmakologi, farmasi-klinik</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Use an existing Category ID when available.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B12" t="str">
+        <v>category_name</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Use category_id or category_name</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Klinis, Farmakologi, Farmasi Klinik or a new Category name</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Use an existing Category name or type a new one to create it during import.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B13" t="str">
+        <v>sub_category_id</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Use sub_category_id or sub_category_name</v>
+      </c>
+      <c r="D13" t="str">
+        <v>klinis-kardiovaskular-hipertensi, klinis-kardiovaskular-gagal-jantung, klinis-respiratori-asma, farmakologi-antibiotik, farmakologi-nsaid, farmasi-klinik-perhitungan-dosis, farmasi-klinik-interaksi-obat</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Must belong to the selected category_id.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B14" t="str">
+        <v>sub_category_name</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Use sub_category_id or sub_category_name</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Kardiovaskular - Hipertensi, Kardiovaskular - Gagal Jantung, Respiratori - Asma, Antibiotik, NSAID, Perhitungan Dosis, Interaksi Obat or a new Sub-category name</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Use an existing Sub-category name or type a new one to create it during import.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B15" t="str">
+        <v>question_text</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Any text</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Question prompt shown to students.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B16" t="str">
+        <v>option_a</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Any text</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Answer option A.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B17" t="str">
+        <v>option_b</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Any text</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Answer option B.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B18" t="str">
+        <v>option_c</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Any text</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Answer option C.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B19" t="str">
+        <v>option_d</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Any text</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Answer option D.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B20" t="str">
+        <v>option_e</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Only when correct_option is E</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Any text or blank</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Leave blank when this question only has A-D options.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B21" t="str">
+        <v>correct_option</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D21" t="str">
+        <v>A, B, C, D, E</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Must match one filled option column.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B22" t="str">
+        <v>explanation</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Any text</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Shown in the review or discussion flow.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B23" t="str">
+        <v>video_url</v>
+      </c>
+      <c r="C23" t="str">
+        <v>No</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Valid URL or blank</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Optional supporting video URL.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B24" t="str">
+        <v>access_level</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D24" t="str">
+        <v>free, premium</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Controls who can access this Question.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>questions</v>
+      </c>
+      <c r="B25" t="str">
+        <v>status</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D25" t="str">
+        <v>draft, published, unpublished</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Published Try-outs need published Questions.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B26" t="str">
+        <v>category_id</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D26" t="str">
+        <v>klinis</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Klinis</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B27" t="str">
+        <v>sub_category_id</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D27" t="str">
+        <v>klinis-kardiovaskular-hipertensi</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Kardiovaskular - Hipertensi under category_id klinis</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B28" t="str">
+        <v>sub_category_id</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D28" t="str">
+        <v>klinis-kardiovaskular-gagal-jantung</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Kardiovaskular - Gagal Jantung under category_id klinis</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B29" t="str">
+        <v>sub_category_id</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D29" t="str">
+        <v>klinis-respiratori-asma</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Respiratori - Asma under category_id klinis</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B30" t="str">
+        <v>category_id</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D30" t="str">
+        <v>farmakologi</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Farmakologi</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B31" t="str">
+        <v>sub_category_id</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D31" t="str">
+        <v>farmakologi-antibiotik</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Antibiotik under category_id farmakologi</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B32" t="str">
+        <v>sub_category_id</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D32" t="str">
+        <v>farmakologi-nsaid</v>
+      </c>
+      <c r="E32" t="str">
+        <v>NSAID under category_id farmakologi</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B33" t="str">
+        <v>category_id</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D33" t="str">
+        <v>farmasi-klinik</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Farmasi Klinik</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B34" t="str">
+        <v>sub_category_id</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D34" t="str">
+        <v>farmasi-klinik-perhitungan-dosis</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Perhitungan Dosis under category_id farmasi-klinik</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B35" t="str">
+        <v>sub_category_id</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D35" t="str">
+        <v>farmasi-klinik-interaksi-obat</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Interaksi Obat under category_id farmasi-klinik</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E35"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add topic-level taxonomy management
</commit_message>
<xml_diff>
--- a/docs/ilmorax-tryout-sample.xlsx
+++ b/docs/ilmorax-tryout-sample.xlsx
@@ -465,7 +465,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:S3"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -473,17 +473,19 @@
     <col min="4" max="4" width="15.83203125" customWidth="1"/>
     <col min="5" max="5" width="17.83203125" customWidth="1"/>
     <col min="6" max="6" width="19.83203125" customWidth="1"/>
-    <col min="7" max="7" width="44.83203125" customWidth="1"/>
-    <col min="8" max="8" width="29.83203125" customWidth="1"/>
-    <col min="9" max="9" width="33.83203125" customWidth="1"/>
-    <col min="10" max="10" width="26.83203125" customWidth="1"/>
-    <col min="11" max="11" width="27.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="16.83203125" customWidth="1"/>
-    <col min="14" max="14" width="72.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="44.83203125" customWidth="1"/>
+    <col min="10" max="10" width="29.83203125" customWidth="1"/>
+    <col min="11" max="11" width="33.83203125" customWidth="1"/>
+    <col min="12" max="12" width="26.83203125" customWidth="1"/>
+    <col min="13" max="13" width="27.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="72.83203125" customWidth="1"/>
     <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,36 +508,42 @@
         <v>sub_category_name</v>
       </c>
       <c r="G1" t="str">
+        <v>topic_id</v>
+      </c>
+      <c r="H1" t="str">
+        <v>topic_name</v>
+      </c>
+      <c r="I1" t="str">
         <v>question_text</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>option_a</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>option_b</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>option_c</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>option_d</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>option_e</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>correct_option</v>
       </c>
-      <c r="N1" t="str">
+      <c r="P1" t="str">
         <v>explanation</v>
       </c>
-      <c r="O1" t="str">
+      <c r="Q1" t="str">
         <v>video_url</v>
       </c>
-      <c r="P1" t="str">
+      <c r="R1" t="str">
         <v>access_level</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="S1" t="str">
         <v>status</v>
       </c>
     </row>
@@ -559,36 +567,42 @@
         <v>Antibiotik</v>
       </c>
       <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>Antibiotik</v>
+      </c>
+      <c r="I2" t="str">
         <v>Mekanisme kerja penisilin adalah:</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>Menghambat sintesis protein</v>
       </c>
-      <c r="I2" t="str">
+      <c r="K2" t="str">
         <v>Menghambat sintesis dinding sel</v>
       </c>
-      <c r="J2" t="str">
+      <c r="L2" t="str">
         <v>Menghambat replikasi DNA</v>
       </c>
-      <c r="K2" t="str">
+      <c r="M2" t="str">
         <v>Menghambat sintesis folat</v>
       </c>
-      <c r="L2" t="str">
+      <c r="N2" t="str">
         <v/>
       </c>
-      <c r="M2" t="str">
+      <c r="O2" t="str">
         <v>B</v>
       </c>
-      <c r="N2" t="str">
+      <c r="P2" t="str">
         <v>Penisilin menghambat sintesis dinding sel bakteri dengan mengikat protein pengikat penisilin.</v>
       </c>
-      <c r="O2" t="str">
+      <c r="Q2" t="str">
         <v/>
       </c>
-      <c r="P2" t="str">
+      <c r="R2" t="str">
         <v>free</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="S2" t="str">
         <v>draft</v>
       </c>
     </row>
@@ -612,49 +626,55 @@
         <v>NSAID</v>
       </c>
       <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>NSAID</v>
+      </c>
+      <c r="I3" t="str">
         <v>NSAID yang paling selektif terhadap COX-2:</v>
       </c>
-      <c r="H3" t="str">
+      <c r="J3" t="str">
         <v>Ibuprofen</v>
       </c>
-      <c r="I3" t="str">
+      <c r="K3" t="str">
         <v>Celecoxib</v>
       </c>
-      <c r="J3" t="str">
+      <c r="L3" t="str">
         <v>Aspirin</v>
       </c>
-      <c r="K3" t="str">
+      <c r="M3" t="str">
         <v>Diklofenak</v>
       </c>
-      <c r="L3" t="str">
+      <c r="N3" t="str">
         <v/>
       </c>
-      <c r="M3" t="str">
+      <c r="O3" t="str">
         <v>B</v>
       </c>
-      <c r="N3" t="str">
+      <c r="P3" t="str">
         <v>Celecoxib adalah NSAID selektif COX-2 yang menurunkan risiko gangguan gastrointestinal.</v>
       </c>
-      <c r="O3" t="str">
+      <c r="Q3" t="str">
         <v/>
       </c>
-      <c r="P3" t="str">
+      <c r="R3" t="str">
         <v>free</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="S3" t="str">
         <v>draft</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E43"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="19.83203125" customWidth="1"/>
@@ -878,7 +898,7 @@
         <v>Use sub_category_id or sub_category_name</v>
       </c>
       <c r="D13" t="str">
-        <v>klinis-kardiovaskular-hipertensi, klinis-kardiovaskular-gagal-jantung, klinis-respiratori-asma, farmakologi-antibiotik, farmakologi-nsaid, farmasi-klinik-perhitungan-dosis, farmasi-klinik-interaksi-obat</v>
+        <v>klinis-kardiovaskular, klinis-respiratori, farmakologi-antibiotik, farmakologi-nsaid, farmasi-klinik-perhitungan-dosis, farmasi-klinik-interaksi-obat</v>
       </c>
       <c r="E13" t="str">
         <v>Must belong to the selected category_id.</v>
@@ -895,7 +915,7 @@
         <v>Use sub_category_id or sub_category_name</v>
       </c>
       <c r="D14" t="str">
-        <v>Kardiovaskular - Hipertensi, Kardiovaskular - Gagal Jantung, Respiratori - Asma, Antibiotik, NSAID, Perhitungan Dosis, Interaksi Obat or a new Sub-category name</v>
+        <v>Kardiovaskular, Respiratori, Antibiotik, NSAID, Perhitungan Dosis, Interaksi Obat or a new Sub-category name</v>
       </c>
       <c r="E14" t="str">
         <v>Use an existing Sub-category name or type a new one to create it during import.</v>
@@ -906,16 +926,16 @@
         <v>questions</v>
       </c>
       <c r="B15" t="str">
-        <v>question_text</v>
+        <v>topic_id</v>
       </c>
       <c r="C15" t="str">
-        <v>Yes</v>
+        <v>Use topic_id or topic_name</v>
       </c>
       <c r="D15" t="str">
-        <v>Any text</v>
+        <v>klinis-kardiovaskular-hipertensi, klinis-kardiovaskular-gagal-jantung, klinis-respiratori-asma, farmakologi-antibiotik-antibiotik, farmakologi-nsaid-nsaid, farmasi-klinik-perhitungan-dosis-perhitungan-dosis, farmasi-klinik-interaksi-obat-interaksi-obat</v>
       </c>
       <c r="E15" t="str">
-        <v>Question prompt shown to students.</v>
+        <v>Must belong to the selected sub_category_id.</v>
       </c>
     </row>
     <row r="16">
@@ -923,16 +943,16 @@
         <v>questions</v>
       </c>
       <c r="B16" t="str">
-        <v>option_a</v>
+        <v>topic_name</v>
       </c>
       <c r="C16" t="str">
-        <v>Yes</v>
+        <v>Use topic_id or topic_name</v>
       </c>
       <c r="D16" t="str">
-        <v>Any text</v>
+        <v>Hipertensi, Gagal Jantung, Asma, Antibiotik, NSAID, Perhitungan Dosis, Interaksi Obat or a new Topic name</v>
       </c>
       <c r="E16" t="str">
-        <v>Answer option A.</v>
+        <v>Use an existing Topic name under the selected Sub-category or type a new one to create it during import.</v>
       </c>
     </row>
     <row r="17">
@@ -940,7 +960,7 @@
         <v>questions</v>
       </c>
       <c r="B17" t="str">
-        <v>option_b</v>
+        <v>question_text</v>
       </c>
       <c r="C17" t="str">
         <v>Yes</v>
@@ -949,7 +969,7 @@
         <v>Any text</v>
       </c>
       <c r="E17" t="str">
-        <v>Answer option B.</v>
+        <v>Question prompt shown to students.</v>
       </c>
     </row>
     <row r="18">
@@ -957,7 +977,7 @@
         <v>questions</v>
       </c>
       <c r="B18" t="str">
-        <v>option_c</v>
+        <v>option_a</v>
       </c>
       <c r="C18" t="str">
         <v>Yes</v>
@@ -966,7 +986,7 @@
         <v>Any text</v>
       </c>
       <c r="E18" t="str">
-        <v>Answer option C.</v>
+        <v>Answer option A.</v>
       </c>
     </row>
     <row r="19">
@@ -974,7 +994,7 @@
         <v>questions</v>
       </c>
       <c r="B19" t="str">
-        <v>option_d</v>
+        <v>option_b</v>
       </c>
       <c r="C19" t="str">
         <v>Yes</v>
@@ -983,7 +1003,7 @@
         <v>Any text</v>
       </c>
       <c r="E19" t="str">
-        <v>Answer option D.</v>
+        <v>Answer option B.</v>
       </c>
     </row>
     <row r="20">
@@ -991,16 +1011,16 @@
         <v>questions</v>
       </c>
       <c r="B20" t="str">
-        <v>option_e</v>
+        <v>option_c</v>
       </c>
       <c r="C20" t="str">
-        <v>Only when correct_option is E</v>
+        <v>Yes</v>
       </c>
       <c r="D20" t="str">
-        <v>Any text or blank</v>
+        <v>Any text</v>
       </c>
       <c r="E20" t="str">
-        <v>Leave blank when this question only has A-D options.</v>
+        <v>Answer option C.</v>
       </c>
     </row>
     <row r="21">
@@ -1008,16 +1028,16 @@
         <v>questions</v>
       </c>
       <c r="B21" t="str">
-        <v>correct_option</v>
+        <v>option_d</v>
       </c>
       <c r="C21" t="str">
         <v>Yes</v>
       </c>
       <c r="D21" t="str">
-        <v>A, B, C, D, E</v>
+        <v>Any text</v>
       </c>
       <c r="E21" t="str">
-        <v>Must match one filled option column.</v>
+        <v>Answer option D.</v>
       </c>
     </row>
     <row r="22">
@@ -1025,16 +1045,16 @@
         <v>questions</v>
       </c>
       <c r="B22" t="str">
-        <v>explanation</v>
+        <v>option_e</v>
       </c>
       <c r="C22" t="str">
-        <v>Yes</v>
+        <v>Only when correct_option is E</v>
       </c>
       <c r="D22" t="str">
-        <v>Any text</v>
+        <v>Any text or blank</v>
       </c>
       <c r="E22" t="str">
-        <v>Shown in the review or discussion flow.</v>
+        <v>Leave blank when this question only has A-D options.</v>
       </c>
     </row>
     <row r="23">
@@ -1042,16 +1062,16 @@
         <v>questions</v>
       </c>
       <c r="B23" t="str">
-        <v>video_url</v>
+        <v>correct_option</v>
       </c>
       <c r="C23" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="D23" t="str">
-        <v>Valid URL or blank</v>
+        <v>A, B, C, D, E</v>
       </c>
       <c r="E23" t="str">
-        <v>Optional supporting video URL.</v>
+        <v>Must match one filled option column.</v>
       </c>
     </row>
     <row r="24">
@@ -1059,16 +1079,16 @@
         <v>questions</v>
       </c>
       <c r="B24" t="str">
-        <v>access_level</v>
+        <v>explanation</v>
       </c>
       <c r="C24" t="str">
         <v>Yes</v>
       </c>
       <c r="D24" t="str">
-        <v>free, premium</v>
+        <v>Any text</v>
       </c>
       <c r="E24" t="str">
-        <v>Controls who can access this Question.</v>
+        <v>Shown in the review or discussion flow.</v>
       </c>
     </row>
     <row r="25">
@@ -1076,50 +1096,50 @@
         <v>questions</v>
       </c>
       <c r="B25" t="str">
-        <v>status</v>
+        <v>video_url</v>
       </c>
       <c r="C25" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="D25" t="str">
-        <v>draft, published, unpublished</v>
+        <v>Valid URL or blank</v>
       </c>
       <c r="E25" t="str">
-        <v>Published Try-outs need published Questions.</v>
+        <v>Optional supporting video URL.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>reference</v>
+        <v>questions</v>
       </c>
       <c r="B26" t="str">
-        <v>category_id</v>
+        <v>access_level</v>
       </c>
       <c r="C26" t="str">
-        <v>Reference</v>
+        <v>Yes</v>
       </c>
       <c r="D26" t="str">
-        <v>klinis</v>
+        <v>free, premium</v>
       </c>
       <c r="E26" t="str">
-        <v>Klinis</v>
+        <v>Controls who can access this Question.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>reference</v>
+        <v>questions</v>
       </c>
       <c r="B27" t="str">
-        <v>sub_category_id</v>
+        <v>status</v>
       </c>
       <c r="C27" t="str">
-        <v>Reference</v>
+        <v>Yes</v>
       </c>
       <c r="D27" t="str">
-        <v>klinis-kardiovaskular-hipertensi</v>
+        <v>draft, published, unpublished</v>
       </c>
       <c r="E27" t="str">
-        <v>Kardiovaskular - Hipertensi under category_id klinis</v>
+        <v>Published Try-outs need published Questions.</v>
       </c>
     </row>
     <row r="28">
@@ -1127,16 +1147,16 @@
         <v>reference</v>
       </c>
       <c r="B28" t="str">
-        <v>sub_category_id</v>
+        <v>category_id</v>
       </c>
       <c r="C28" t="str">
         <v>Reference</v>
       </c>
       <c r="D28" t="str">
-        <v>klinis-kardiovaskular-gagal-jantung</v>
+        <v>klinis</v>
       </c>
       <c r="E28" t="str">
-        <v>Kardiovaskular - Gagal Jantung under category_id klinis</v>
+        <v>Klinis</v>
       </c>
     </row>
     <row r="29">
@@ -1150,10 +1170,10 @@
         <v>Reference</v>
       </c>
       <c r="D29" t="str">
-        <v>klinis-respiratori-asma</v>
+        <v>klinis-kardiovaskular</v>
       </c>
       <c r="E29" t="str">
-        <v>Respiratori - Asma under category_id klinis</v>
+        <v>Kardiovaskular under category_id klinis</v>
       </c>
     </row>
     <row r="30">
@@ -1161,16 +1181,16 @@
         <v>reference</v>
       </c>
       <c r="B30" t="str">
-        <v>category_id</v>
+        <v>topic_id</v>
       </c>
       <c r="C30" t="str">
         <v>Reference</v>
       </c>
       <c r="D30" t="str">
-        <v>farmakologi</v>
+        <v>klinis-kardiovaskular-hipertensi</v>
       </c>
       <c r="E30" t="str">
-        <v>Farmakologi</v>
+        <v>Hipertensi under sub_category_id klinis-kardiovaskular</v>
       </c>
     </row>
     <row r="31">
@@ -1178,16 +1198,16 @@
         <v>reference</v>
       </c>
       <c r="B31" t="str">
-        <v>sub_category_id</v>
+        <v>topic_id</v>
       </c>
       <c r="C31" t="str">
         <v>Reference</v>
       </c>
       <c r="D31" t="str">
-        <v>farmakologi-antibiotik</v>
+        <v>klinis-kardiovaskular-gagal-jantung</v>
       </c>
       <c r="E31" t="str">
-        <v>Antibiotik under category_id farmakologi</v>
+        <v>Gagal Jantung under sub_category_id klinis-kardiovaskular</v>
       </c>
     </row>
     <row r="32">
@@ -1201,10 +1221,10 @@
         <v>Reference</v>
       </c>
       <c r="D32" t="str">
-        <v>farmakologi-nsaid</v>
+        <v>klinis-respiratori</v>
       </c>
       <c r="E32" t="str">
-        <v>NSAID under category_id farmakologi</v>
+        <v>Respiratori under category_id klinis</v>
       </c>
     </row>
     <row r="33">
@@ -1212,16 +1232,16 @@
         <v>reference</v>
       </c>
       <c r="B33" t="str">
-        <v>category_id</v>
+        <v>topic_id</v>
       </c>
       <c r="C33" t="str">
         <v>Reference</v>
       </c>
       <c r="D33" t="str">
-        <v>farmasi-klinik</v>
+        <v>klinis-respiratori-asma</v>
       </c>
       <c r="E33" t="str">
-        <v>Farmasi Klinik</v>
+        <v>Asma under sub_category_id klinis-respiratori</v>
       </c>
     </row>
     <row r="34">
@@ -1229,16 +1249,16 @@
         <v>reference</v>
       </c>
       <c r="B34" t="str">
-        <v>sub_category_id</v>
+        <v>category_id</v>
       </c>
       <c r="C34" t="str">
         <v>Reference</v>
       </c>
       <c r="D34" t="str">
-        <v>farmasi-klinik-perhitungan-dosis</v>
+        <v>farmakologi</v>
       </c>
       <c r="E34" t="str">
-        <v>Perhitungan Dosis under category_id farmasi-klinik</v>
+        <v>Farmakologi</v>
       </c>
     </row>
     <row r="35">
@@ -1252,15 +1272,151 @@
         <v>Reference</v>
       </c>
       <c r="D35" t="str">
+        <v>farmakologi-antibiotik</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Antibiotik under category_id farmakologi</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B36" t="str">
+        <v>topic_id</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D36" t="str">
+        <v>farmakologi-antibiotik-antibiotik</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Antibiotik under sub_category_id farmakologi-antibiotik</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B37" t="str">
+        <v>sub_category_id</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D37" t="str">
+        <v>farmakologi-nsaid</v>
+      </c>
+      <c r="E37" t="str">
+        <v>NSAID under category_id farmakologi</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B38" t="str">
+        <v>topic_id</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D38" t="str">
+        <v>farmakologi-nsaid-nsaid</v>
+      </c>
+      <c r="E38" t="str">
+        <v>NSAID under sub_category_id farmakologi-nsaid</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B39" t="str">
+        <v>category_id</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D39" t="str">
+        <v>farmasi-klinik</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Farmasi Klinik</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B40" t="str">
+        <v>sub_category_id</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D40" t="str">
+        <v>farmasi-klinik-perhitungan-dosis</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Perhitungan Dosis under category_id farmasi-klinik</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B41" t="str">
+        <v>topic_id</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D41" t="str">
+        <v>farmasi-klinik-perhitungan-dosis-perhitungan-dosis</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Perhitungan Dosis under sub_category_id farmasi-klinik-perhitungan-dosis</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B42" t="str">
+        <v>sub_category_id</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D42" t="str">
         <v>farmasi-klinik-interaksi-obat</v>
       </c>
-      <c r="E35" t="str">
+      <c r="E42" t="str">
         <v>Interaksi Obat under category_id farmasi-klinik</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>reference</v>
+      </c>
+      <c r="B43" t="str">
+        <v>topic_id</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Reference</v>
+      </c>
+      <c r="D43" t="str">
+        <v>farmasi-klinik-interaksi-obat-interaksi-obat</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Interaksi Obat under sub_category_id farmasi-klinik-interaksi-obat</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E43"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>